<commit_message>
added new changes for update and authorize test steps
</commit_message>
<xml_diff>
--- a/src/test/resources/paypal_multi_order_with_items.xlsx
+++ b/src/test/resources/paypal_multi_order_with_items.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="113">
   <si>
     <t>order_id</t>
   </si>
@@ -171,6 +171,9 @@
   </si>
   <si>
     <t>INV_9010</t>
+  </si>
+  <si>
+    <t>ORDER_1_AUTH</t>
   </si>
   <si>
     <t>item_name</t>
@@ -378,19 +381,13 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10.5"/>
-      <color rgb="FF2C2E2F"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -855,139 +852,138 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1334,7 +1330,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="25.8888888888889" customWidth="1"/>
@@ -1395,7 +1391,7 @@
       <c r="A2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
       <c r="C2" t="s">
@@ -1798,6 +1794,47 @@
         <v>24</v>
       </c>
       <c r="M11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>19</v>
+      </c>
+      <c r="H12" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" t="s">
+        <v>22</v>
+      </c>
+      <c r="K12" t="s">
+        <v>23</v>
+      </c>
+      <c r="L12" t="s">
+        <v>24</v>
+      </c>
+      <c r="M12" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1810,7 +1847,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1818,37 +1855,37 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F1" t="s">
         <v>9</v>
       </c>
       <c r="G1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -1856,37 +1893,37 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
         <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -1894,37 +1931,37 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F3" t="s">
         <v>22</v>
       </c>
       <c r="G3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -1932,37 +1969,37 @@
         <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F4" t="s">
         <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -1970,37 +2007,37 @@
         <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F5" t="s">
         <v>22</v>
       </c>
       <c r="G5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -2008,37 +2045,37 @@
         <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
         <v>22</v>
       </c>
       <c r="G6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -2046,37 +2083,37 @@
         <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
         <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -2084,37 +2121,37 @@
         <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F8" t="s">
         <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L8" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2122,37 +2159,37 @@
         <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
         <v>22</v>
       </c>
       <c r="G9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2160,37 +2197,37 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
         <v>22</v>
       </c>
       <c r="G10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L10" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2198,37 +2235,37 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
         <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -2236,37 +2273,37 @@
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
         <v>22</v>
       </c>
       <c r="G12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -2274,37 +2311,37 @@
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
         <v>22</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L13" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:12">
@@ -2312,37 +2349,37 @@
         <v>37</v>
       </c>
       <c r="B14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F14" t="s">
         <v>22</v>
       </c>
       <c r="G14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -2350,37 +2387,37 @@
         <v>37</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
         <v>22</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L15" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:12">
@@ -2388,37 +2425,37 @@
         <v>40</v>
       </c>
       <c r="B16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E16" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F16" t="s">
         <v>22</v>
       </c>
       <c r="G16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H16" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J16" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K16" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:12">
@@ -2426,37 +2463,37 @@
         <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E17" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F17" t="s">
         <v>22</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L17" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:12">
@@ -2464,37 +2501,37 @@
         <v>42</v>
       </c>
       <c r="B18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F18" t="s">
         <v>22</v>
       </c>
       <c r="G18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L18" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:12">
@@ -2502,37 +2539,37 @@
         <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F19" t="s">
         <v>22</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:12">
@@ -2540,37 +2577,37 @@
         <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D20" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F20" t="s">
         <v>22</v>
       </c>
       <c r="G20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="J20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="K20" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:12">
@@ -2578,60 +2615,136 @@
         <v>45</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D21" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
         <v>22</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="I21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K21" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="L21" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" t="s">
+        <v>61</v>
+      </c>
+      <c r="F22" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
         <v>58</v>
       </c>
-      <c r="D22" t="s">
+      <c r="C23" t="s">
         <v>59</v>
       </c>
-      <c r="E22" t="s">
+      <c r="D23" t="s">
         <v>60</v>
       </c>
-      <c r="F22" t="s">
-        <v>22</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="E23" t="s">
+        <v>61</v>
+      </c>
+      <c r="F23" t="s">
+        <v>22</v>
+      </c>
+      <c r="G23" t="s">
+        <v>62</v>
+      </c>
+      <c r="H23" t="s">
+        <v>63</v>
+      </c>
+      <c r="I23" t="s">
+        <v>64</v>
+      </c>
+      <c r="J23" t="s">
+        <v>65</v>
+      </c>
+      <c r="K23" t="s">
+        <v>66</v>
+      </c>
+      <c r="L23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s">
         <v>71</v>
+      </c>
+      <c r="F24" t="s">
+        <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>72</v>
+      </c>
+      <c r="H24" t="s">
+        <v>63</v>
+      </c>
+      <c r="I24" t="s">
+        <v>73</v>
+      </c>
+      <c r="J24" t="s">
+        <v>74</v>
+      </c>
+      <c r="K24" t="s">
+        <v>66</v>
+      </c>
+      <c r="L24" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>